<commit_message>
fix(bom): sync 94 rows between FA-273 NEW MFG and MFG ECN MASTER SHEET
</commit_message>
<xml_diff>
--- a/BOM/MFG ECN MASTER SHEET.xlsx
+++ b/BOM/MFG ECN MASTER SHEET.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\MASTER SHEET\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Darshan Details\Internship Faith Automation\Projects\Spare Part Tracking\SpareTrack\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18B5C97B-F07E-442B-A007-2082467447E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4879D27C-D9AB-4AC6-A2BE-3CBFC75646BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="583" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="571" uniqueCount="41">
   <si>
     <t>Project Code</t>
   </si>
@@ -420,7 +420,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -475,16 +475,13 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="7" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -779,18 +776,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="C3:I100"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="C3:I98"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="3" max="4" width="20.28515625" customWidth="1"/>
-    <col min="5" max="5" width="29.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.5703125" customWidth="1"/>
-    <col min="7" max="7" width="16.85546875" customWidth="1"/>
-    <col min="8" max="8" width="15.42578125" customWidth="1"/>
+    <col min="3" max="4" width="20.33203125" customWidth="1"/>
+    <col min="5" max="5" width="29.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.5546875" customWidth="1"/>
+    <col min="7" max="7" width="16.88671875" customWidth="1"/>
+    <col min="8" max="8" width="15.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="3:9" ht="15.75" thickBot="1"/>
-    <row r="4" spans="3:9" ht="21.75" thickBot="1">
+    <row r="3" spans="3:9" ht="15" thickBot="1"/>
+    <row r="4" spans="3:9" ht="21.6" thickBot="1">
       <c r="C4" s="7" t="s">
         <v>0</v>
       </c>
@@ -823,10 +820,10 @@
       <c r="E5" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="F5" s="22" t="s">
+      <c r="F5" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="G5" s="22" t="s">
+      <c r="G5" s="21" t="s">
         <v>12</v>
       </c>
       <c r="H5" s="12" t="s">
@@ -846,10 +843,10 @@
       <c r="E6" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="F6" s="23" t="s">
+      <c r="F6" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="G6" s="23" t="s">
+      <c r="G6" s="22" t="s">
         <v>15</v>
       </c>
       <c r="H6" s="6" t="s">
@@ -869,10 +866,10 @@
       <c r="E7" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="F7" s="23" t="s">
+      <c r="F7" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="G7" s="23" t="s">
+      <c r="G7" s="22" t="s">
         <v>8</v>
       </c>
       <c r="H7" s="6" t="s">
@@ -892,10 +889,10 @@
       <c r="E8" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="F8" s="23" t="s">
-        <v>16</v>
-      </c>
-      <c r="G8" s="23" t="s">
+      <c r="F8" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="G8" s="22" t="s">
         <v>8</v>
       </c>
       <c r="H8" s="6" t="s">
@@ -915,10 +912,10 @@
       <c r="E9" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="F9" s="23" t="s">
+      <c r="F9" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="G9" s="23" t="s">
+      <c r="G9" s="22" t="s">
         <v>8</v>
       </c>
       <c r="H9" s="6" t="s">
@@ -938,10 +935,10 @@
       <c r="E10" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="F10" s="23" t="s">
+      <c r="F10" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="G10" s="23" t="s">
+      <c r="G10" s="22" t="s">
         <v>8</v>
       </c>
       <c r="H10" s="6" t="s">
@@ -961,10 +958,10 @@
       <c r="E11" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="F11" s="23" t="s">
+      <c r="F11" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="G11" s="23" t="s">
+      <c r="G11" s="22" t="s">
         <v>8</v>
       </c>
       <c r="H11" s="6" t="s">
@@ -984,10 +981,10 @@
       <c r="E12" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="F12" s="23" t="s">
-        <v>16</v>
-      </c>
-      <c r="G12" s="23" t="s">
+      <c r="F12" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="G12" s="22" t="s">
         <v>8</v>
       </c>
       <c r="H12" s="6" t="s">
@@ -1007,10 +1004,10 @@
       <c r="E13" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="F13" s="23" t="s">
+      <c r="F13" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="G13" s="23" t="s">
+      <c r="G13" s="22" t="s">
         <v>12</v>
       </c>
       <c r="H13" s="6" t="s">
@@ -1030,10 +1027,10 @@
       <c r="E14" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="F14" s="23" t="s">
+      <c r="F14" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="G14" s="23" t="s">
+      <c r="G14" s="22" t="s">
         <v>15</v>
       </c>
       <c r="H14" s="6" t="s">
@@ -1053,10 +1050,10 @@
       <c r="E15" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="F15" s="23" t="s">
+      <c r="F15" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="G15" s="23" t="s">
+      <c r="G15" s="22" t="s">
         <v>8</v>
       </c>
       <c r="H15" s="6" t="s">
@@ -1076,10 +1073,10 @@
       <c r="E16" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="F16" s="23" t="s">
-        <v>16</v>
-      </c>
-      <c r="G16" s="23" t="s">
+      <c r="F16" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="G16" s="22" t="s">
         <v>8</v>
       </c>
       <c r="H16" s="6" t="s">
@@ -1099,10 +1096,10 @@
       <c r="E17" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="F17" s="23" t="s">
+      <c r="F17" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="G17" s="23" t="s">
+      <c r="G17" s="22" t="s">
         <v>8</v>
       </c>
       <c r="H17" s="6" t="s">
@@ -1122,10 +1119,10 @@
       <c r="E18" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="F18" s="23" t="s">
+      <c r="F18" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="G18" s="23" t="s">
+      <c r="G18" s="22" t="s">
         <v>8</v>
       </c>
       <c r="H18" s="6" t="s">
@@ -1145,10 +1142,10 @@
       <c r="E19" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="F19" s="23" t="s">
+      <c r="F19" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="G19" s="23" t="s">
+      <c r="G19" s="22" t="s">
         <v>8</v>
       </c>
       <c r="H19" s="6" t="s">
@@ -1168,10 +1165,10 @@
       <c r="E20" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="F20" s="23" t="s">
-        <v>16</v>
-      </c>
-      <c r="G20" s="23" t="s">
+      <c r="F20" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="G20" s="22" t="s">
         <v>8</v>
       </c>
       <c r="H20" s="6" t="s">
@@ -1191,10 +1188,10 @@
       <c r="E21" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="F21" s="23" t="s">
+      <c r="F21" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="G21" s="23" t="s">
+      <c r="G21" s="22" t="s">
         <v>12</v>
       </c>
       <c r="H21" s="6" t="s">
@@ -1214,10 +1211,10 @@
       <c r="E22" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="F22" s="23" t="s">
+      <c r="F22" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="G22" s="23" t="s">
+      <c r="G22" s="22" t="s">
         <v>15</v>
       </c>
       <c r="H22" s="6" t="s">
@@ -1237,10 +1234,10 @@
       <c r="E23" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="F23" s="23" t="s">
+      <c r="F23" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="G23" s="23" t="s">
+      <c r="G23" s="22" t="s">
         <v>8</v>
       </c>
       <c r="H23" s="6" t="s">
@@ -1260,10 +1257,10 @@
       <c r="E24" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="F24" s="23" t="s">
-        <v>16</v>
-      </c>
-      <c r="G24" s="23" t="s">
+      <c r="F24" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="G24" s="22" t="s">
         <v>8</v>
       </c>
       <c r="H24" s="6" t="s">
@@ -1283,10 +1280,10 @@
       <c r="E25" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="F25" s="23" t="s">
+      <c r="F25" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="G25" s="23" t="s">
+      <c r="G25" s="22" t="s">
         <v>8</v>
       </c>
       <c r="H25" s="6" t="s">
@@ -1306,10 +1303,10 @@
       <c r="E26" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="F26" s="23" t="s">
+      <c r="F26" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="G26" s="23" t="s">
+      <c r="G26" s="22" t="s">
         <v>8</v>
       </c>
       <c r="H26" s="6" t="s">
@@ -1329,10 +1326,10 @@
       <c r="E27" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="F27" s="23" t="s">
+      <c r="F27" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="G27" s="23" t="s">
+      <c r="G27" s="22" t="s">
         <v>8</v>
       </c>
       <c r="H27" s="6" t="s">
@@ -1352,10 +1349,10 @@
       <c r="E28" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="F28" s="23" t="s">
-        <v>16</v>
-      </c>
-      <c r="G28" s="23" t="s">
+      <c r="F28" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="G28" s="22" t="s">
         <v>8</v>
       </c>
       <c r="H28" s="6" t="s">
@@ -1375,10 +1372,10 @@
       <c r="E29" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="F29" s="23" t="s">
+      <c r="F29" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="G29" s="23" t="s">
+      <c r="G29" s="22" t="s">
         <v>12</v>
       </c>
       <c r="H29" s="6" t="s">
@@ -1398,10 +1395,10 @@
       <c r="E30" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="F30" s="23" t="s">
+      <c r="F30" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="G30" s="23" t="s">
+      <c r="G30" s="22" t="s">
         <v>15</v>
       </c>
       <c r="H30" s="6" t="s">
@@ -1421,10 +1418,10 @@
       <c r="E31" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="F31" s="23" t="s">
+      <c r="F31" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="G31" s="23" t="s">
+      <c r="G31" s="22" t="s">
         <v>8</v>
       </c>
       <c r="H31" s="6" t="s">
@@ -1444,10 +1441,10 @@
       <c r="E32" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="F32" s="23" t="s">
-        <v>16</v>
-      </c>
-      <c r="G32" s="23" t="s">
+      <c r="F32" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="G32" s="22" t="s">
         <v>8</v>
       </c>
       <c r="H32" s="6" t="s">
@@ -1467,10 +1464,10 @@
       <c r="E33" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="F33" s="23" t="s">
+      <c r="F33" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="G33" s="23" t="s">
+      <c r="G33" s="22" t="s">
         <v>8</v>
       </c>
       <c r="H33" s="6" t="s">
@@ -1490,10 +1487,10 @@
       <c r="E34" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="F34" s="23" t="s">
+      <c r="F34" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="G34" s="23" t="s">
+      <c r="G34" s="22" t="s">
         <v>8</v>
       </c>
       <c r="H34" s="6" t="s">
@@ -1513,10 +1510,10 @@
       <c r="E35" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="F35" s="23" t="s">
+      <c r="F35" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="G35" s="23" t="s">
+      <c r="G35" s="22" t="s">
         <v>8</v>
       </c>
       <c r="H35" s="6" t="s">
@@ -1531,21 +1528,21 @@
         <v>18</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="E36" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="F36" s="23" t="s">
-        <v>16</v>
-      </c>
-      <c r="G36" s="23" t="s">
-        <v>8</v>
+        <v>23</v>
+      </c>
+      <c r="E36" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="F36" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="G36" s="22" t="s">
+        <v>6</v>
       </c>
       <c r="H36" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="I36" s="15">
+        <v>36</v>
+      </c>
+      <c r="I36" s="16">
         <v>1</v>
       </c>
     </row>
@@ -1559,11 +1556,11 @@
       <c r="E37" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F37" s="23" t="s">
-        <v>16</v>
-      </c>
-      <c r="G37" s="23" t="s">
-        <v>6</v>
+      <c r="F37" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="G37" s="22" t="s">
+        <v>8</v>
       </c>
       <c r="H37" s="6" t="s">
         <v>36</v>
@@ -1582,11 +1579,11 @@
       <c r="E38" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F38" s="23" t="s">
-        <v>16</v>
-      </c>
-      <c r="G38" s="23" t="s">
-        <v>8</v>
+      <c r="F38" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="G38" s="22" t="s">
+        <v>10</v>
       </c>
       <c r="H38" s="6" t="s">
         <v>36</v>
@@ -1605,11 +1602,11 @@
       <c r="E39" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F39" s="23" t="s">
-        <v>16</v>
-      </c>
-      <c r="G39" s="23" t="s">
-        <v>10</v>
+      <c r="F39" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="G39" s="22" t="s">
+        <v>11</v>
       </c>
       <c r="H39" s="6" t="s">
         <v>36</v>
@@ -1628,11 +1625,11 @@
       <c r="E40" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F40" s="23" t="s">
-        <v>16</v>
-      </c>
-      <c r="G40" s="23" t="s">
-        <v>11</v>
+      <c r="F40" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="G40" s="22" t="s">
+        <v>12</v>
       </c>
       <c r="H40" s="6" t="s">
         <v>36</v>
@@ -1651,11 +1648,11 @@
       <c r="E41" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F41" s="23" t="s">
-        <v>16</v>
-      </c>
-      <c r="G41" s="23" t="s">
-        <v>12</v>
+      <c r="F41" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="G41" s="22" t="s">
+        <v>13</v>
       </c>
       <c r="H41" s="6" t="s">
         <v>36</v>
@@ -1674,11 +1671,11 @@
       <c r="E42" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F42" s="23" t="s">
-        <v>16</v>
-      </c>
-      <c r="G42" s="23" t="s">
-        <v>13</v>
+      <c r="F42" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="G42" s="22" t="s">
+        <v>14</v>
       </c>
       <c r="H42" s="6" t="s">
         <v>36</v>
@@ -1697,11 +1694,11 @@
       <c r="E43" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F43" s="23" t="s">
-        <v>16</v>
-      </c>
-      <c r="G43" s="23" t="s">
-        <v>14</v>
+      <c r="F43" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="G43" s="22" t="s">
+        <v>15</v>
       </c>
       <c r="H43" s="6" t="s">
         <v>36</v>
@@ -1720,11 +1717,11 @@
       <c r="E44" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F44" s="23" t="s">
-        <v>16</v>
-      </c>
-      <c r="G44" s="23" t="s">
-        <v>15</v>
+      <c r="F44" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="G44" s="22" t="s">
+        <v>16</v>
       </c>
       <c r="H44" s="6" t="s">
         <v>36</v>
@@ -1743,11 +1740,11 @@
       <c r="E45" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F45" s="23" t="s">
-        <v>16</v>
-      </c>
-      <c r="G45" s="23" t="s">
-        <v>16</v>
+      <c r="F45" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="G45" s="22" t="s">
+        <v>17</v>
       </c>
       <c r="H45" s="6" t="s">
         <v>36</v>
@@ -1766,11 +1763,11 @@
       <c r="E46" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F46" s="23" t="s">
-        <v>16</v>
-      </c>
-      <c r="G46" s="23" t="s">
-        <v>17</v>
+      <c r="F46" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="G46" s="22" t="s">
+        <v>19</v>
       </c>
       <c r="H46" s="6" t="s">
         <v>36</v>
@@ -1786,19 +1783,19 @@
       <c r="D47" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="E47" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="F47" s="23" t="s">
-        <v>16</v>
-      </c>
-      <c r="G47" s="23" t="s">
+      <c r="E47" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="F47" s="22" t="s">
         <v>19</v>
       </c>
+      <c r="G47" s="22" t="s">
+        <v>6</v>
+      </c>
       <c r="H47" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="I47" s="16">
+      <c r="I47" s="17">
         <v>1</v>
       </c>
     </row>
@@ -1812,11 +1809,11 @@
       <c r="E48" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="F48" s="23" t="s">
+      <c r="F48" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="G48" s="23" t="s">
-        <v>6</v>
+      <c r="G48" s="22" t="s">
+        <v>8</v>
       </c>
       <c r="H48" s="6" t="s">
         <v>36</v>
@@ -1835,11 +1832,11 @@
       <c r="E49" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="F49" s="23" t="s">
+      <c r="F49" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="G49" s="23" t="s">
-        <v>8</v>
+      <c r="G49" s="22" t="s">
+        <v>10</v>
       </c>
       <c r="H49" s="6" t="s">
         <v>36</v>
@@ -1858,11 +1855,11 @@
       <c r="E50" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="F50" s="23" t="s">
+      <c r="F50" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="G50" s="23" t="s">
-        <v>10</v>
+      <c r="G50" s="22" t="s">
+        <v>11</v>
       </c>
       <c r="H50" s="6" t="s">
         <v>36</v>
@@ -1881,11 +1878,11 @@
       <c r="E51" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="F51" s="23" t="s">
+      <c r="F51" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="G51" s="23" t="s">
-        <v>11</v>
+      <c r="G51" s="22" t="s">
+        <v>12</v>
       </c>
       <c r="H51" s="6" t="s">
         <v>36</v>
@@ -1904,11 +1901,11 @@
       <c r="E52" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="F52" s="23" t="s">
+      <c r="F52" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="G52" s="23" t="s">
-        <v>12</v>
+      <c r="G52" s="22" t="s">
+        <v>13</v>
       </c>
       <c r="H52" s="6" t="s">
         <v>36</v>
@@ -1927,11 +1924,11 @@
       <c r="E53" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="F53" s="23" t="s">
+      <c r="F53" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="G53" s="23" t="s">
-        <v>13</v>
+      <c r="G53" s="22" t="s">
+        <v>14</v>
       </c>
       <c r="H53" s="6" t="s">
         <v>36</v>
@@ -1950,11 +1947,11 @@
       <c r="E54" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="F54" s="23" t="s">
+      <c r="F54" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="G54" s="23" t="s">
-        <v>14</v>
+      <c r="G54" s="22" t="s">
+        <v>15</v>
       </c>
       <c r="H54" s="6" t="s">
         <v>36</v>
@@ -1973,11 +1970,11 @@
       <c r="E55" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="F55" s="23" t="s">
+      <c r="F55" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="G55" s="23" t="s">
-        <v>15</v>
+      <c r="G55" s="22" t="s">
+        <v>16</v>
       </c>
       <c r="H55" s="6" t="s">
         <v>36</v>
@@ -1996,11 +1993,11 @@
       <c r="E56" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="F56" s="23" t="s">
+      <c r="F56" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="G56" s="23" t="s">
-        <v>16</v>
+      <c r="G56" s="22" t="s">
+        <v>17</v>
       </c>
       <c r="H56" s="6" t="s">
         <v>36</v>
@@ -2016,19 +2013,19 @@
       <c r="D57" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="E57" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="F57" s="23" t="s">
-        <v>19</v>
-      </c>
-      <c r="G57" s="23" t="s">
-        <v>17</v>
+      <c r="E57" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="F57" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="G57" s="22" t="s">
+        <v>6</v>
       </c>
       <c r="H57" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="I57" s="17">
+        <v>7</v>
+      </c>
+      <c r="I57" s="16">
         <v>1</v>
       </c>
     </row>
@@ -2042,11 +2039,11 @@
       <c r="E58" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F58" s="23" t="s">
+      <c r="F58" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="G58" s="23" t="s">
-        <v>6</v>
+      <c r="G58" s="22" t="s">
+        <v>8</v>
       </c>
       <c r="H58" s="6" t="s">
         <v>7</v>
@@ -2065,11 +2062,11 @@
       <c r="E59" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F59" s="23" t="s">
+      <c r="F59" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="G59" s="23" t="s">
-        <v>8</v>
+      <c r="G59" s="22" t="s">
+        <v>10</v>
       </c>
       <c r="H59" s="6" t="s">
         <v>7</v>
@@ -2088,11 +2085,11 @@
       <c r="E60" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F60" s="23" t="s">
+      <c r="F60" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="G60" s="23" t="s">
-        <v>10</v>
+      <c r="G60" s="22" t="s">
+        <v>11</v>
       </c>
       <c r="H60" s="6" t="s">
         <v>7</v>
@@ -2111,11 +2108,11 @@
       <c r="E61" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F61" s="23" t="s">
+      <c r="F61" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="G61" s="23" t="s">
-        <v>11</v>
+      <c r="G61" s="22" t="s">
+        <v>12</v>
       </c>
       <c r="H61" s="6" t="s">
         <v>7</v>
@@ -2134,11 +2131,11 @@
       <c r="E62" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F62" s="23" t="s">
+      <c r="F62" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="G62" s="23" t="s">
-        <v>12</v>
+      <c r="G62" s="22" t="s">
+        <v>13</v>
       </c>
       <c r="H62" s="6" t="s">
         <v>7</v>
@@ -2157,11 +2154,11 @@
       <c r="E63" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F63" s="23" t="s">
+      <c r="F63" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="G63" s="23" t="s">
-        <v>13</v>
+      <c r="G63" s="22" t="s">
+        <v>14</v>
       </c>
       <c r="H63" s="6" t="s">
         <v>7</v>
@@ -2180,11 +2177,11 @@
       <c r="E64" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F64" s="23" t="s">
+      <c r="F64" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="G64" s="23" t="s">
-        <v>14</v>
+      <c r="G64" s="22" t="s">
+        <v>15</v>
       </c>
       <c r="H64" s="6" t="s">
         <v>7</v>
@@ -2203,14 +2200,14 @@
       <c r="E65" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F65" s="23" t="s">
-        <v>20</v>
-      </c>
-      <c r="G65" s="23" t="s">
-        <v>15</v>
+      <c r="F65" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="G65" s="22" t="s">
+        <v>6</v>
       </c>
       <c r="H65" s="6" t="s">
-        <v>7</v>
+        <v>37</v>
       </c>
       <c r="I65" s="16">
         <v>1</v>
@@ -2226,11 +2223,11 @@
       <c r="E66" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F66" s="23" t="s">
-        <v>16</v>
-      </c>
-      <c r="G66" s="23" t="s">
-        <v>6</v>
+      <c r="F66" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="G66" s="22" t="s">
+        <v>10</v>
       </c>
       <c r="H66" s="6" t="s">
         <v>37</v>
@@ -2249,11 +2246,11 @@
       <c r="E67" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F67" s="23" t="s">
-        <v>16</v>
-      </c>
-      <c r="G67" s="23" t="s">
-        <v>8</v>
+      <c r="F67" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="G67" s="22" t="s">
+        <v>11</v>
       </c>
       <c r="H67" s="6" t="s">
         <v>37</v>
@@ -2272,11 +2269,11 @@
       <c r="E68" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F68" s="23" t="s">
-        <v>16</v>
-      </c>
-      <c r="G68" s="23" t="s">
-        <v>10</v>
+      <c r="F68" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="G68" s="22" t="s">
+        <v>12</v>
       </c>
       <c r="H68" s="6" t="s">
         <v>37</v>
@@ -2295,11 +2292,11 @@
       <c r="E69" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F69" s="23" t="s">
-        <v>16</v>
-      </c>
-      <c r="G69" s="23" t="s">
-        <v>11</v>
+      <c r="F69" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="G69" s="22" t="s">
+        <v>13</v>
       </c>
       <c r="H69" s="6" t="s">
         <v>37</v>
@@ -2318,11 +2315,11 @@
       <c r="E70" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F70" s="23" t="s">
-        <v>16</v>
-      </c>
-      <c r="G70" s="23" t="s">
-        <v>12</v>
+      <c r="F70" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="G70" s="22" t="s">
+        <v>14</v>
       </c>
       <c r="H70" s="6" t="s">
         <v>37</v>
@@ -2341,11 +2338,11 @@
       <c r="E71" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F71" s="23" t="s">
-        <v>16</v>
-      </c>
-      <c r="G71" s="23" t="s">
-        <v>13</v>
+      <c r="F71" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="G71" s="22" t="s">
+        <v>15</v>
       </c>
       <c r="H71" s="6" t="s">
         <v>37</v>
@@ -2364,11 +2361,11 @@
       <c r="E72" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F72" s="23" t="s">
-        <v>16</v>
-      </c>
-      <c r="G72" s="23" t="s">
-        <v>14</v>
+      <c r="F72" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="G72" s="22" t="s">
+        <v>16</v>
       </c>
       <c r="H72" s="6" t="s">
         <v>37</v>
@@ -2387,11 +2384,11 @@
       <c r="E73" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F73" s="23" t="s">
-        <v>16</v>
-      </c>
-      <c r="G73" s="23" t="s">
-        <v>15</v>
+      <c r="F73" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="G73" s="22" t="s">
+        <v>17</v>
       </c>
       <c r="H73" s="6" t="s">
         <v>37</v>
@@ -2410,11 +2407,11 @@
       <c r="E74" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F74" s="23" t="s">
-        <v>16</v>
-      </c>
-      <c r="G74" s="23" t="s">
-        <v>16</v>
+      <c r="F74" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="G74" s="22" t="s">
+        <v>19</v>
       </c>
       <c r="H74" s="6" t="s">
         <v>37</v>
@@ -2430,19 +2427,19 @@
       <c r="D75" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="E75" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="F75" s="23" t="s">
-        <v>16</v>
-      </c>
-      <c r="G75" s="23" t="s">
-        <v>17</v>
+      <c r="E75" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="F75" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="G75" s="22" t="s">
+        <v>6</v>
       </c>
       <c r="H75" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="I75" s="16">
+      <c r="I75" s="17">
         <v>1</v>
       </c>
     </row>
@@ -2453,19 +2450,19 @@
       <c r="D76" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="E76" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="F76" s="23" t="s">
-        <v>16</v>
-      </c>
-      <c r="G76" s="23" t="s">
+      <c r="E76" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="F76" s="22" t="s">
         <v>19</v>
       </c>
+      <c r="G76" s="22" t="s">
+        <v>8</v>
+      </c>
       <c r="H76" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="I76" s="16">
+      <c r="I76" s="17">
         <v>1</v>
       </c>
     </row>
@@ -2479,11 +2476,11 @@
       <c r="E77" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="F77" s="23" t="s">
+      <c r="F77" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="G77" s="23" t="s">
-        <v>6</v>
+      <c r="G77" s="22" t="s">
+        <v>10</v>
       </c>
       <c r="H77" s="6" t="s">
         <v>37</v>
@@ -2502,11 +2499,11 @@
       <c r="E78" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="F78" s="23" t="s">
+      <c r="F78" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="G78" s="23" t="s">
-        <v>8</v>
+      <c r="G78" s="22" t="s">
+        <v>11</v>
       </c>
       <c r="H78" s="6" t="s">
         <v>37</v>
@@ -2525,11 +2522,11 @@
       <c r="E79" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="F79" s="23" t="s">
+      <c r="F79" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="G79" s="23" t="s">
-        <v>10</v>
+      <c r="G79" s="22" t="s">
+        <v>12</v>
       </c>
       <c r="H79" s="6" t="s">
         <v>37</v>
@@ -2548,11 +2545,11 @@
       <c r="E80" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="F80" s="23" t="s">
+      <c r="F80" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="G80" s="23" t="s">
-        <v>11</v>
+      <c r="G80" s="22" t="s">
+        <v>13</v>
       </c>
       <c r="H80" s="6" t="s">
         <v>37</v>
@@ -2571,11 +2568,11 @@
       <c r="E81" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="F81" s="23" t="s">
+      <c r="F81" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="G81" s="23" t="s">
-        <v>12</v>
+      <c r="G81" s="22" t="s">
+        <v>14</v>
       </c>
       <c r="H81" s="6" t="s">
         <v>37</v>
@@ -2594,11 +2591,11 @@
       <c r="E82" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="F82" s="23" t="s">
+      <c r="F82" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="G82" s="23" t="s">
-        <v>13</v>
+      <c r="G82" s="22" t="s">
+        <v>15</v>
       </c>
       <c r="H82" s="6" t="s">
         <v>37</v>
@@ -2617,11 +2614,11 @@
       <c r="E83" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="F83" s="23" t="s">
+      <c r="F83" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="G83" s="23" t="s">
-        <v>14</v>
+      <c r="G83" s="22" t="s">
+        <v>16</v>
       </c>
       <c r="H83" s="6" t="s">
         <v>37</v>
@@ -2640,11 +2637,11 @@
       <c r="E84" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="F84" s="23" t="s">
+      <c r="F84" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="G84" s="23" t="s">
-        <v>15</v>
+      <c r="G84" s="22" t="s">
+        <v>17</v>
       </c>
       <c r="H84" s="6" t="s">
         <v>37</v>
@@ -2660,19 +2657,19 @@
       <c r="D85" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="E85" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="F85" s="23" t="s">
-        <v>19</v>
-      </c>
-      <c r="G85" s="23" t="s">
-        <v>16</v>
+      <c r="E85" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="F85" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="G85" s="22" t="s">
+        <v>6</v>
       </c>
       <c r="H85" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="I85" s="17">
+        <v>9</v>
+      </c>
+      <c r="I85" s="16">
         <v>1</v>
       </c>
     </row>
@@ -2683,19 +2680,19 @@
       <c r="D86" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="E86" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="F86" s="23" t="s">
-        <v>19</v>
-      </c>
-      <c r="G86" s="23" t="s">
-        <v>17</v>
+      <c r="E86" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="F86" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="G86" s="22" t="s">
+        <v>8</v>
       </c>
       <c r="H86" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="I86" s="17">
+        <v>9</v>
+      </c>
+      <c r="I86" s="16">
         <v>1</v>
       </c>
     </row>
@@ -2709,11 +2706,11 @@
       <c r="E87" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F87" s="23" t="s">
+      <c r="F87" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="G87" s="23" t="s">
-        <v>6</v>
+      <c r="G87" s="22" t="s">
+        <v>10</v>
       </c>
       <c r="H87" s="6" t="s">
         <v>9</v>
@@ -2732,11 +2729,11 @@
       <c r="E88" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F88" s="23" t="s">
+      <c r="F88" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="G88" s="23" t="s">
-        <v>8</v>
+      <c r="G88" s="22" t="s">
+        <v>11</v>
       </c>
       <c r="H88" s="6" t="s">
         <v>9</v>
@@ -2755,11 +2752,11 @@
       <c r="E89" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F89" s="23" t="s">
+      <c r="F89" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="G89" s="23" t="s">
-        <v>10</v>
+      <c r="G89" s="22" t="s">
+        <v>12</v>
       </c>
       <c r="H89" s="6" t="s">
         <v>9</v>
@@ -2778,11 +2775,11 @@
       <c r="E90" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F90" s="23" t="s">
+      <c r="F90" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="G90" s="23" t="s">
-        <v>11</v>
+      <c r="G90" s="22" t="s">
+        <v>13</v>
       </c>
       <c r="H90" s="6" t="s">
         <v>9</v>
@@ -2801,11 +2798,11 @@
       <c r="E91" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F91" s="23" t="s">
+      <c r="F91" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="G91" s="23" t="s">
-        <v>12</v>
+      <c r="G91" s="22" t="s">
+        <v>14</v>
       </c>
       <c r="H91" s="6" t="s">
         <v>9</v>
@@ -2824,11 +2821,11 @@
       <c r="E92" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F92" s="23" t="s">
+      <c r="F92" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="G92" s="23" t="s">
-        <v>13</v>
+      <c r="G92" s="22" t="s">
+        <v>15</v>
       </c>
       <c r="H92" s="6" t="s">
         <v>9</v>
@@ -2842,19 +2839,19 @@
         <v>18</v>
       </c>
       <c r="D93" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E93" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="F93" s="23" t="s">
-        <v>20</v>
-      </c>
-      <c r="G93" s="23" t="s">
-        <v>14</v>
+        <v>34</v>
+      </c>
+      <c r="F93" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="G93" s="22" t="s">
+        <v>8</v>
       </c>
       <c r="H93" s="6" t="s">
-        <v>9</v>
+        <v>39</v>
       </c>
       <c r="I93" s="16">
         <v>1</v>
@@ -2865,19 +2862,19 @@
         <v>18</v>
       </c>
       <c r="D94" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E94" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="F94" s="23" t="s">
-        <v>20</v>
-      </c>
-      <c r="G94" s="23" t="s">
-        <v>15</v>
+        <v>35</v>
+      </c>
+      <c r="F94" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="G94" s="22" t="s">
+        <v>8</v>
       </c>
       <c r="H94" s="6" t="s">
-        <v>9</v>
+        <v>40</v>
       </c>
       <c r="I94" s="16">
         <v>1</v>
@@ -2888,21 +2885,21 @@
         <v>18</v>
       </c>
       <c r="D95" s="6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E95" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="F95" s="23" t="s">
-        <v>38</v>
-      </c>
-      <c r="G95" s="23" t="s">
-        <v>8</v>
+        <v>29</v>
+      </c>
+      <c r="F95" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="G95" s="22" t="s">
+        <v>13</v>
       </c>
       <c r="H95" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="I95" s="18">
+      <c r="I95" s="16">
         <v>1</v>
       </c>
     </row>
@@ -2911,21 +2908,21 @@
         <v>18</v>
       </c>
       <c r="D96" s="6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E96" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="F96" s="23" t="s">
-        <v>38</v>
-      </c>
-      <c r="G96" s="23" t="s">
-        <v>8</v>
+        <v>29</v>
+      </c>
+      <c r="F96" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="G96" s="22" t="s">
+        <v>13</v>
       </c>
       <c r="H96" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="I96" s="18">
+      <c r="I96" s="16">
         <v>1</v>
       </c>
     </row>
@@ -2937,30 +2934,30 @@
         <v>25</v>
       </c>
       <c r="E97" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="F97" s="23" t="s">
+        <v>27</v>
+      </c>
+      <c r="F97" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="G97" s="23" t="s">
+      <c r="G97" s="22" t="s">
         <v>13</v>
       </c>
       <c r="H97" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="I97" s="18">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="98" spans="3:9" ht="21">
-      <c r="C98" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D98" s="6" t="s">
+      <c r="I97" s="16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="98" spans="3:9" ht="21.6" thickBot="1">
+      <c r="C98" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D98" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="E98" s="4" t="s">
-        <v>29</v>
+      <c r="E98" s="19" t="s">
+        <v>27</v>
       </c>
       <c r="F98" s="23" t="s">
         <v>11</v>
@@ -2968,56 +2965,10 @@
       <c r="G98" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="H98" s="6" t="s">
+      <c r="H98" s="18" t="s">
         <v>40</v>
       </c>
-      <c r="I98" s="18">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="99" spans="3:9" ht="21">
-      <c r="C99" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D99" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="E99" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="F99" s="23" t="s">
-        <v>11</v>
-      </c>
-      <c r="G99" s="23" t="s">
-        <v>13</v>
-      </c>
-      <c r="H99" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="I99" s="18">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="100" spans="3:9" ht="21.75" thickBot="1">
-      <c r="C100" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D100" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="E100" s="20" t="s">
-        <v>27</v>
-      </c>
-      <c r="F100" s="24" t="s">
-        <v>11</v>
-      </c>
-      <c r="G100" s="24" t="s">
-        <v>13</v>
-      </c>
-      <c r="H100" s="19" t="s">
-        <v>40</v>
-      </c>
-      <c r="I100" s="21">
+      <c r="I98" s="20">
         <v>1</v>
       </c>
     </row>
@@ -3025,7 +2976,7 @@
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="F5:G100" numberStoredAsText="1"/>
+    <ignoredError sqref="F5:G35 F66:G98 F36:G65" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>